<commit_message>
docs(example): regenerate the exports on the merged branches
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqoocMczx3spPPqhrRpAE5
</commit_message>
<xml_diff>
--- a/docs/example/coretax-export.xlsx
+++ b/docs/example/coretax-export.xlsx
@@ -225,10 +225,10 @@
   </numFmts>
   <fonts count="7">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -239,31 +239,31 @@
       <color rgb="00FFFFFF"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <charset val="1"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="12"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <sz val="12"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>

</xml_diff>

<commit_message>
docs(example): regenerate the exports with centred table cells
The three PDFs now show each row's cells centred against a wrapped name,
and every workbook carries the vertical centring.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqoocMczx3spPPqhrRpAE5
</commit_message>
<xml_diff>
--- a/docs/example/coretax-export.xlsx
+++ b/docs/example/coretax-export.xlsx
@@ -399,8 +399,8 @@
       <alignment wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" quotePrefix="false" pivotButton="false"/>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyAlignment="false">
-      <alignment/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyAlignment="true">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyAlignment="false">
       <alignment/>
@@ -6137,122 +6137,122 @@
   <dimension ref="A1"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="19" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s">
+      <c r="A3" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="K3" t="s">
+      <c r="K3" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="L3" t="s">
+      <c r="L3" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="M3" t="s">
+      <c r="M3" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="N3" t="s">
+      <c r="N3" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="O3" t="s">
+      <c r="O3" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="P3" t="s">
+      <c r="P3" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="Q3" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="R3" t="s">
+      <c r="R3" s="19" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4">
+      <c r="A4" s="19">
         <v>1</v>
       </c>
       <c r="B4" s="24">
         <v>46306</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="J4" t="s">
+      <c r="J4" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="K4" t="s">
+      <c r="K4" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="L4" t="s">
+      <c r="L4" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="M4" t="s">
+      <c r="M4" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="N4" t="s">
+      <c r="N4" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="O4" t="s">
+      <c r="O4" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="P4" t="s">
+      <c r="P4" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="Q4" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="R4" t="s">
+      <c r="R4" s="19" t="s">
         <v>46</v>
       </c>
     </row>
@@ -6265,331 +6265,331 @@
   <dimension ref="A1"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="19" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
+      <c r="A2" s="19">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="19">
         <v>2400000</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="19">
         <v>2</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="19">
         <v>240000</v>
       </c>
-      <c r="I2">
+      <c r="I2" s="19">
         <v>4560000</v>
       </c>
-      <c r="J2">
+      <c r="J2" s="19">
         <v>4180000</v>
       </c>
-      <c r="K2">
+      <c r="K2" s="19">
         <v>12</v>
       </c>
-      <c r="L2">
+      <c r="L2" s="19">
         <v>501600</v>
       </c>
-      <c r="M2">
+      <c r="M2" s="19">
         <v>0</v>
       </c>
-      <c r="N2">
+      <c r="N2" s="19">
         <v>0</v>
       </c>
-      <c r="O2" t="s">
+      <c r="O2" s="19" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3">
+      <c r="A3" s="19">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="19">
         <v>65000</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="19">
         <v>10</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="19">
         <v>32500</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="19">
         <v>617500</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="19">
         <v>566041.67</v>
       </c>
-      <c r="K3">
+      <c r="K3" s="19">
         <v>12</v>
       </c>
-      <c r="L3">
+      <c r="L3" s="19">
         <v>67925</v>
       </c>
-      <c r="M3">
+      <c r="M3" s="19">
         <v>0</v>
       </c>
-      <c r="N3">
+      <c r="N3" s="19">
         <v>0</v>
       </c>
-      <c r="O3" t="s">
+      <c r="O3" s="19" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4">
+      <c r="A4" s="19">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="19">
         <v>525000</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="19">
         <v>6</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="19">
         <v>157500</v>
       </c>
-      <c r="I4">
+      <c r="I4" s="19">
         <v>2992500</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="19">
         <v>2743125</v>
       </c>
-      <c r="K4">
+      <c r="K4" s="19">
         <v>12</v>
       </c>
-      <c r="L4">
+      <c r="L4" s="19">
         <v>329175</v>
       </c>
-      <c r="M4">
+      <c r="M4" s="19">
         <v>0</v>
       </c>
-      <c r="N4">
+      <c r="N4" s="19">
         <v>0</v>
       </c>
-      <c r="O4" t="s">
+      <c r="O4" s="19" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5">
+      <c r="A5" s="19">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="19">
         <v>1690000</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="19">
         <v>4</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="19">
         <v>338000</v>
       </c>
-      <c r="I5">
+      <c r="I5" s="19">
         <v>6422000</v>
       </c>
-      <c r="J5">
+      <c r="J5" s="19">
         <v>5886833.33</v>
       </c>
-      <c r="K5">
+      <c r="K5" s="19">
         <v>12</v>
       </c>
-      <c r="L5">
+      <c r="L5" s="19">
         <v>706420</v>
       </c>
-      <c r="M5">
+      <c r="M5" s="19">
         <v>0</v>
       </c>
-      <c r="N5">
+      <c r="N5" s="19">
         <v>0</v>
       </c>
-      <c r="O5" t="s">
+      <c r="O5" s="19" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6">
+      <c r="A6" s="19">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="19">
         <v>24000</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="19">
         <v>100</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="19">
         <v>120000</v>
       </c>
-      <c r="I6">
+      <c r="I6" s="19">
         <v>2280000</v>
       </c>
-      <c r="J6">
+      <c r="J6" s="19">
         <v>2090000</v>
       </c>
-      <c r="K6">
+      <c r="K6" s="19">
         <v>12</v>
       </c>
-      <c r="L6">
+      <c r="L6" s="19">
         <v>250800</v>
       </c>
-      <c r="M6">
+      <c r="M6" s="19">
         <v>0</v>
       </c>
-      <c r="N6">
+      <c r="N6" s="19">
         <v>0</v>
       </c>
-      <c r="O6" t="s">
+      <c r="O6" s="19" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7">
+      <c r="A7" s="19">
         <v>6</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="19">
         <v>750000</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="19">
         <v>1</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="19">
         <v>0</v>
       </c>
-      <c r="I7">
+      <c r="I7" s="19">
         <v>750000</v>
       </c>
-      <c r="J7">
+      <c r="J7" s="19">
         <v>687500</v>
       </c>
-      <c r="K7">
+      <c r="K7" s="19">
         <v>12</v>
       </c>
-      <c r="L7">
+      <c r="L7" s="19">
         <v>82500</v>
       </c>
-      <c r="M7">
+      <c r="M7" s="19">
         <v>0</v>
       </c>
-      <c r="N7">
+      <c r="N7" s="19">
         <v>0</v>
       </c>
-      <c r="O7" t="s">
+      <c r="O7" s="19" t="s">
         <v>37</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(example): show the delivery note Address and Notes
The example sale now saves one Surat Jalan note and sends its last line
to another dock, so the example prints both a saved note and a default.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqoocMczx3spPPqhrRpAE5
</commit_message>
<xml_diff>
--- a/docs/example/coretax-export.xlsx
+++ b/docs/example/coretax-export.xlsx
@@ -20,10 +20,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
   <si>
-    <t>NPWP Penjual</t>
+    <t>0987654321098765</t>
   </si>
   <si>
-    <t>0987654321098765</t>
+    <t>NPWP Penjual</t>
   </si>
   <si>
     <t>Baris</t>
@@ -6138,10 +6138,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="19" t="s">
         <v>0</v>
-      </c>
-      <c r="C1" s="19" t="s">
-        <v>1</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
docs(example): regenerate the exports on the merged v0.35 branches
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqoocMczx3spPPqhrRpAE5
</commit_message>
<xml_diff>
--- a/docs/example/coretax-export.xlsx
+++ b/docs/example/coretax-export.xlsx
@@ -20,10 +20,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
   <si>
-    <t>0987654321098765</t>
+    <t>NPWP Penjual</t>
   </si>
   <si>
-    <t>NPWP Penjual</t>
+    <t>0987654321098765</t>
   </si>
   <si>
     <t>Baris</t>
@@ -6138,10 +6138,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="19" t="s">
         <v>1</v>
-      </c>
-      <c r="C1" s="19" t="s">
-        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>